<commit_message>
KPI actualizado 2026-08-21 16:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001591 - ZITRON COLOMBIA  ARIS MARAMTO.xlsx
+++ b/data/50001591 - ZITRON COLOMBIA  ARIS MARAMTO.xlsx
@@ -159,46 +159,46 @@
     <t>Ingenieria Detalle</t>
   </si>
   <si>
+    <t>1217120302071407</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingenieria Basica Motor </t>
+  </si>
+  <si>
+    <t>Propuesta Motor ot 4394</t>
+  </si>
+  <si>
+    <t>1217119129757861</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Plano Preliminar  OT 4394</t>
+  </si>
+  <si>
+    <t>1217117619809521</t>
+  </si>
+  <si>
+    <t>Reservas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva Alabes OT 4394 ,Reserva rodete  OT 4394  </t>
+  </si>
+  <si>
+    <t>1217119120448611</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva Alabes OT 4394 </t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe OT 4394,Reservas</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1217120302071407</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingenieria Basica Motor </t>
-  </si>
-  <si>
-    <t>Propuesta Motor ot 4394</t>
-  </si>
-  <si>
-    <t>1217119129757861</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Plano Preliminar  OT 4394</t>
-  </si>
-  <si>
-    <t>1217117619809521</t>
-  </si>
-  <si>
-    <t>Reservas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva Alabes OT 4394 ,Reserva rodete  OT 4394  </t>
-  </si>
-  <si>
-    <t>1217119120448611</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva Alabes OT 4394 </t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe OT 4394,Reservas</t>
   </si>
   <si>
     <t>1217119227894752</t>
@@ -1945,9 +1945,11 @@
       <c r="B8" s="5">
         <v>46237.57017201389</v>
       </c>
-      <c r="C8" s="6"/>
+      <c r="C8" s="5">
+        <v>46255.6631494676</v>
+      </c>
       <c r="D8" s="5">
-        <v>46252.553109479166</v>
+        <v>46255.663162129626</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>40</v>
@@ -1982,24 +1984,28 @@
       <c r="Q8" s="6"/>
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="12" t="s">
-        <v>42</v>
+      <c r="T8" s="6">
+        <v>1</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="9">
         <v>46237.77875482639</v>
       </c>
-      <c r="C9" s="10"/>
+      <c r="C9" s="9">
+        <v>46255.663131863424</v>
+      </c>
       <c r="D9" s="9">
-        <v>46241.205332928235</v>
+        <v>46255.66314921297</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>26</v>
@@ -2032,7 +2038,7 @@
         <v>37</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Q9" s="9">
         <v>46240</v>
@@ -2044,15 +2050,15 @@
         <v>33</v>
       </c>
       <c r="T9" s="10">
-        <v>0</v>
-      </c>
-      <c r="U9" s="12" t="s">
-        <v>42</v>
+        <v>1</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="5">
         <v>46237.570322175925</v>
@@ -2097,7 +2103,7 @@
         <v>37</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Q10" s="5">
         <v>46241</v>
@@ -2117,7 +2123,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B11" s="9">
         <v>46237.57017664352</v>
@@ -2127,7 +2133,7 @@
         <v>46237.786044988425</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>25</v>
@@ -2151,7 +2157,7 @@
         <v>26</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>26</v>
@@ -2164,7 +2170,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="5">
         <v>46237.5703287963</v>
@@ -2174,16 +2180,16 @@
         <v>46240.19889532407</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I12" s="5">
         <v>46238</v>
@@ -2201,13 +2207,13 @@
         <v>26</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>37</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q12" s="5">
         <v>46239</v>
@@ -2222,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="U12" s="12" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -2243,10 +2249,10 @@
         <v>26</v>
       </c>
       <c r="G13" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I13" s="9">
         <v>46238</v>
@@ -2264,7 +2270,7 @@
         <v>26</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>37</v>
@@ -2285,7 +2291,7 @@
         <v>0</v>
       </c>
       <c r="U13" s="12" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -2353,10 +2359,10 @@
         <v>26</v>
       </c>
       <c r="G15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I15" s="9">
         <v>46274</v>
@@ -2416,10 +2422,10 @@
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I16" s="5">
         <v>46274</v>
@@ -2479,10 +2485,10 @@
         <v>26</v>
       </c>
       <c r="G17" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I17" s="9">
         <v>46274</v>
@@ -2542,10 +2548,10 @@
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I18" s="5">
         <v>46274</v>
@@ -2594,12 +2600,14 @@
       <c r="B19" s="9">
         <v>46237.579729386576</v>
       </c>
-      <c r="C19" s="10"/>
+      <c r="C19" s="9">
+        <v>46255.66323561342</v>
+      </c>
       <c r="D19" s="9">
-        <v>46246.200580046294</v>
+        <v>46255.663251018515</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
@@ -2629,7 +2637,7 @@
         <v>60</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>77</v>
@@ -2644,10 +2652,10 @@
         <v>33</v>
       </c>
       <c r="T19" s="10">
-        <v>0</v>
-      </c>
-      <c r="U19" s="11" t="s">
-        <v>66</v>
+        <v>1</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
@@ -3443,9 +3451,11 @@
       <c r="B34" s="5">
         <v>46237.580047511576</v>
       </c>
-      <c r="C34" s="6"/>
+      <c r="C34" s="5">
+        <v>46255.66337146991</v>
+      </c>
       <c r="D34" s="5">
-        <v>46239.56952222223</v>
+        <v>46255.66338287037</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>123</v>
@@ -3493,10 +3503,10 @@
         <v>65</v>
       </c>
       <c r="T34" s="6">
-        <v>0</v>
-      </c>
-      <c r="U34" s="11" t="s">
-        <v>66</v>
+        <v>1</v>
+      </c>
+      <c r="U34" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3506,9 +3516,11 @@
       <c r="B35" s="9">
         <v>46237.58011546296</v>
       </c>
-      <c r="C35" s="10"/>
+      <c r="C35" s="9">
+        <v>46255.663279155095</v>
+      </c>
       <c r="D35" s="9">
-        <v>46254.16999688657</v>
+        <v>46255.66328059028</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>77</v>
@@ -3541,7 +3553,7 @@
         <v>123</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>128</v>
@@ -3559,9 +3571,11 @@
       <c r="B36" s="5">
         <v>46237.580208009254</v>
       </c>
-      <c r="C36" s="6"/>
+      <c r="C36" s="5">
+        <v>46255.663358391204</v>
+      </c>
       <c r="D36" s="5">
-        <v>46240.824531493054</v>
+        <v>46255.66335965278</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>130</v>
@@ -3612,9 +3626,11 @@
       <c r="B37" s="9">
         <v>46237.58026069445</v>
       </c>
-      <c r="C37" s="10"/>
+      <c r="C37" s="9">
+        <v>46255.66334458333</v>
+      </c>
       <c r="D37" s="9">
-        <v>46240.82452775463</v>
+        <v>46255.66334568287</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>133</v>
@@ -3779,7 +3795,7 @@
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46252.604395</v>
+        <v>46255.66349910879</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>144</v>
@@ -3829,8 +3845,8 @@
       <c r="T40" s="6">
         <v>0</v>
       </c>
-      <c r="U40" s="11" t="s">
-        <v>66</v>
+      <c r="U40" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -5341,7 +5357,7 @@
         <v>217</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="P67" s="10" t="s">
         <v>221</v>
@@ -5434,7 +5450,7 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46239.61757642361</v>
+        <v>46255.66337329861</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>225</v>
@@ -5484,8 +5500,8 @@
       <c r="T69" s="10">
         <v>0</v>
       </c>
-      <c r="U69" s="11" t="s">
-        <v>66</v>
+      <c r="U69" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5553,10 +5569,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I71" s="9">
         <v>46308</v>
@@ -5616,10 +5632,10 @@
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I72" s="5">
         <v>46308</v>
@@ -5669,10 +5685,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I73" s="9">
         <v>46308</v>
@@ -5722,10 +5738,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I74" s="5">
         <v>46308</v>
@@ -5775,10 +5791,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I75" s="9">
         <v>46308</v>
@@ -5828,10 +5844,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I76" s="5">
         <v>46315</v>
@@ -5891,10 +5907,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I77" s="9">
         <v>46315</v>
@@ -5944,10 +5960,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I78" s="5">
         <v>46315</v>
@@ -5997,10 +6013,10 @@
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H79" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I79" s="9">
         <v>46315</v>
@@ -6050,10 +6066,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I80" s="5">
         <v>46315</v>
@@ -6103,10 +6119,10 @@
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H81" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H81" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I81" s="9">
         <v>46316</v>
@@ -6166,10 +6182,10 @@
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I82" s="5">
         <v>46316</v>
@@ -6219,10 +6235,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H83" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H83" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I83" s="9">
         <v>46316</v>
@@ -6272,10 +6288,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H84" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I84" s="5">
         <v>46316</v>
@@ -6325,10 +6341,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H85" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H85" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I85" s="9">
         <v>46316</v>
@@ -6378,10 +6394,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H86" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I86" s="5">
         <v>46317</v>
@@ -6441,10 +6457,10 @@
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H87" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H87" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I87" s="9">
         <v>46317</v>
@@ -6494,10 +6510,10 @@
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H88" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H88" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I88" s="5">
         <v>46317</v>
@@ -6547,10 +6563,10 @@
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H89" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H89" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I89" s="9">
         <v>46317</v>
@@ -6600,10 +6616,10 @@
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H90" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H90" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I90" s="5">
         <v>46317</v>
@@ -6653,10 +6669,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H91" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H91" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I91" s="9">
         <v>46318</v>
@@ -6716,10 +6732,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H92" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H92" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I92" s="5">
         <v>46318</v>
@@ -6769,10 +6785,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H93" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H93" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I93" s="9">
         <v>46318</v>
@@ -6822,10 +6838,10 @@
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H94" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H94" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I94" s="5">
         <v>46318</v>
@@ -6875,10 +6891,10 @@
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H95" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H95" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I95" s="9">
         <v>46323</v>
@@ -6928,10 +6944,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I96" s="5">
         <v>46321</v>
@@ -6991,10 +7007,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H97" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H97" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I97" s="9">
         <v>46321</v>
@@ -7044,10 +7060,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H98" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H98" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I98" s="5">
         <v>46321</v>
@@ -7097,10 +7113,10 @@
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H99" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H99" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I99" s="9">
         <v>46321</v>
@@ -7150,10 +7166,10 @@
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H100" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H100" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I100" s="5">
         <v>46321</v>
@@ -7203,10 +7219,10 @@
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H101" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H101" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I101" s="9">
         <v>46323</v>
@@ -7266,10 +7282,10 @@
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H102" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H102" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I102" s="5">
         <v>46323</v>
@@ -7319,10 +7335,10 @@
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H103" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H103" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I103" s="9">
         <v>46323</v>
@@ -7372,10 +7388,10 @@
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H104" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H104" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I104" s="5">
         <v>46323</v>
@@ -7425,10 +7441,10 @@
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H105" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H105" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I105" s="9">
         <v>46323</v>
@@ -7800,10 +7816,10 @@
         <v>26</v>
       </c>
       <c r="G112" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H112" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H112" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I112" s="5">
         <v>46325</v>
@@ -7863,10 +7879,10 @@
         <v>26</v>
       </c>
       <c r="G113" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H113" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H113" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I113" s="9">
         <v>46325</v>
@@ -7916,10 +7932,10 @@
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H114" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H114" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I114" s="5">
         <v>46325</v>
@@ -7969,10 +7985,10 @@
         <v>26</v>
       </c>
       <c r="G115" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="H115" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="H115" s="10" t="s">
-        <v>54</v>
       </c>
       <c r="I115" s="9">
         <v>46325</v>
@@ -8022,10 +8038,10 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H116" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="H116" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="I116" s="6"/>
       <c r="J116" s="5">

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-21 16:42 Chile
</commit_message>
<xml_diff>
--- a/data/50001591 - ZITRON COLOMBIA  ARIS MARAMTO.xlsx
+++ b/data/50001591 - ZITRON COLOMBIA  ARIS MARAMTO.xlsx
@@ -231,61 +231,61 @@
     <t>Baja</t>
   </si>
   <si>
+    <t>1217119120468560</t>
+  </si>
+  <si>
+    <t>Propuesta Corte plasma   OT 4394</t>
+  </si>
+  <si>
+    <t>Generacion OC Corte plasma OT  4394</t>
+  </si>
+  <si>
+    <t>1217119120468573</t>
+  </si>
+  <si>
+    <t>Propuesta Fabricación externa   OT 4394</t>
+  </si>
+  <si>
+    <t>Preparacion materiales  OT 4394,Generacion Oc 4394</t>
+  </si>
+  <si>
+    <t>1217119015630774</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta Mecanizado  OT 4394  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC mecanizado  OT 4394 </t>
+  </si>
+  <si>
+    <t>1217117339188565</t>
+  </si>
+  <si>
+    <t>Generación OC Motor OT 4394</t>
+  </si>
+  <si>
+    <t>1217117339188557</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Corte Laser   OT 4394</t>
+  </si>
+  <si>
+    <t>1217119015630789</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricacion corte laser  ot 4394 ,Generación OC corte laser   ot 4394</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1217119120468560</t>
-  </si>
-  <si>
-    <t>Propuesta Corte plasma   OT 4394</t>
-  </si>
-  <si>
-    <t>Generacion OC Corte plasma OT  4394</t>
-  </si>
-  <si>
-    <t>1217119120468573</t>
-  </si>
-  <si>
-    <t>Propuesta Fabricación externa   OT 4394</t>
-  </si>
-  <si>
-    <t>Preparacion materiales  OT 4394,Generacion Oc 4394</t>
-  </si>
-  <si>
-    <t>1217119015630774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta Mecanizado  OT 4394  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC mecanizado  OT 4394 </t>
-  </si>
-  <si>
-    <t>1217117339188565</t>
-  </si>
-  <si>
-    <t>Generación OC Motor OT 4394</t>
-  </si>
-  <si>
-    <t>1217117339188557</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Corte Laser   OT 4394</t>
-  </si>
-  <si>
-    <t>1217119015630789</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricacion corte laser  ot 4394 ,Generación OC corte laser   ot 4394</t>
   </si>
   <si>
     <t>1217119129799398</t>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="9">
-        <v>46239.569350798614</v>
+        <v>46255.715312071756</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>61</v>
@@ -2400,23 +2400,23 @@
       <c r="T15" s="10">
         <v>0</v>
       </c>
-      <c r="U15" s="11" t="s">
-        <v>66</v>
+      <c r="U15" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B16" s="5">
         <v>46237.570353981486</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46239.56934689815</v>
+        <v>46255.71531288195</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2449,7 +2449,7 @@
         <v>63</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Q16" s="5">
         <v>46275</v>
@@ -2463,23 +2463,23 @@
       <c r="T16" s="6">
         <v>0</v>
       </c>
-      <c r="U16" s="11" t="s">
-        <v>66</v>
+      <c r="U16" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B17" s="9">
         <v>46237.570357986115</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46239.5693430324</v>
+        <v>46255.71531201389</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
@@ -2512,7 +2512,7 @@
         <v>63</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Q17" s="9">
         <v>46275</v>
@@ -2526,23 +2526,23 @@
       <c r="T17" s="10">
         <v>0</v>
       </c>
-      <c r="U17" s="11" t="s">
-        <v>66</v>
+      <c r="U17" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="5">
         <v>46237.57036226852</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46239.56933935185</v>
+        <v>46255.715312361106</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
@@ -2575,7 +2575,7 @@
         <v>63</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="Q18" s="5">
         <v>46275</v>
@@ -2589,13 +2589,13 @@
       <c r="T18" s="6">
         <v>0</v>
       </c>
-      <c r="U18" s="11" t="s">
-        <v>66</v>
+      <c r="U18" s="12" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B19" s="9">
         <v>46237.579729386576</v>
@@ -2640,7 +2640,7 @@
         <v>43</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q19" s="9">
         <v>46245</v>
@@ -2660,7 +2660,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" s="5">
         <v>46237.570187731486</v>
@@ -2670,7 +2670,7 @@
         <v>46237.79138571759</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>25</v>
@@ -2694,7 +2694,7 @@
         <v>26</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P20" s="6" t="s">
         <v>26</v>
@@ -2707,7 +2707,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B21" s="9">
         <v>46237.57036725694</v>
@@ -2717,16 +2717,16 @@
         <v>46239.56948452546</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="I21" s="9">
         <v>46276</v>
@@ -2744,13 +2744,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q21" s="9">
         <v>46290</v>
@@ -2765,7 +2765,7 @@
         <v>0</v>
       </c>
       <c r="U21" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
@@ -2786,10 +2786,10 @@
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="I22" s="5">
         <v>46276</v>
@@ -2807,7 +2807,7 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>61</v>
@@ -2824,7 +2824,7 @@
         <v>0</v>
       </c>
       <c r="U22" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -2845,10 +2845,10 @@
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H23" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="I23" s="9">
         <v>46281</v>
@@ -2866,7 +2866,7 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O23" s="10" t="s">
         <v>86</v>
@@ -2883,7 +2883,7 @@
         <v>0</v>
       </c>
       <c r="U23" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -2904,10 +2904,10 @@
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="I24" s="5">
         <v>46276</v>
@@ -2925,7 +2925,7 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>93</v>
@@ -2946,7 +2946,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -2961,16 +2961,16 @@
         <v>46239.56972798611</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="I25" s="9">
         <v>46276</v>
@@ -2991,7 +2991,7 @@
         <v>92</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>95</v>
@@ -3020,10 +3020,10 @@
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="I26" s="5">
         <v>46281</v>
@@ -3044,7 +3044,7 @@
         <v>92</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>98</v>
@@ -3073,10 +3073,10 @@
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="I27" s="9">
         <v>46276</v>
@@ -3094,7 +3094,7 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>101</v>
@@ -3115,7 +3115,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3130,16 +3130,16 @@
         <v>46239.56982333334</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="I28" s="5">
         <v>46276</v>
@@ -3160,7 +3160,7 @@
         <v>100</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>103</v>
@@ -3189,10 +3189,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>83</v>
       </c>
       <c r="I29" s="9">
         <v>46281</v>
@@ -3213,7 +3213,7 @@
         <v>100</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>106</v>
@@ -3263,7 +3263,7 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>111</v>
@@ -3284,7 +3284,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3329,7 +3329,7 @@
         <v>108</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P31" s="10" t="s">
         <v>114</v>
@@ -3485,7 +3485,7 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>126</v>
@@ -3523,7 +3523,7 @@
         <v>46255.66328059028</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
@@ -3608,7 +3608,7 @@
         <v>123</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>131</v>
@@ -3663,7 +3663,7 @@
         <v>123</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="P37" s="10" t="s">
         <v>134</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46252.60439458334</v>
+        <v>46255.71529688657</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>136</v>
@@ -3793,9 +3793,11 @@
       <c r="B40" s="5">
         <v>46237.57046512731</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46255.71516604167</v>
+      </c>
       <c r="D40" s="5">
-        <v>46255.66349910879</v>
+        <v>46255.715192986114</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>144</v>
@@ -3843,10 +3845,10 @@
         <v>65</v>
       </c>
       <c r="T40" s="6">
-        <v>0</v>
-      </c>
-      <c r="U40" s="12" t="s">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="U40" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -3856,9 +3858,11 @@
       <c r="B41" s="9">
         <v>46237.57046940972</v>
       </c>
-      <c r="C41" s="10"/>
+      <c r="C41" s="9">
+        <v>46255.71528109953</v>
+      </c>
       <c r="D41" s="9">
-        <v>46239.57030957176</v>
+        <v>46255.71529815972</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>63</v>
@@ -3906,10 +3910,10 @@
         <v>65</v>
       </c>
       <c r="T41" s="10">
-        <v>0</v>
-      </c>
-      <c r="U41" s="11" t="s">
-        <v>66</v>
+        <v>1</v>
+      </c>
+      <c r="U41" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -3972,7 +3976,7 @@
         <v>0</v>
       </c>
       <c r="U42" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -4294,7 +4298,7 @@
         <v>0</v>
       </c>
       <c r="U48" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -4357,7 +4361,7 @@
         <v>0</v>
       </c>
       <c r="U49" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -4420,7 +4424,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4483,7 +4487,7 @@
         <v>0</v>
       </c>
       <c r="U51" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
@@ -4546,7 +4550,7 @@
         <v>0</v>
       </c>
       <c r="U52" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
@@ -4609,7 +4613,7 @@
         <v>0</v>
       </c>
       <c r="U53" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4701,7 +4705,7 @@
         <v>187</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P55" s="10" t="s">
         <v>193</v>
@@ -4719,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="U55" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4782,7 +4786,7 @@
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4794,7 +4798,7 @@
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46239.57090008102</v>
+        <v>46255.71530028935</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>157</v>
@@ -4847,7 +4851,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46239.570895972225</v>
+        <v>46255.7152974537</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>157</v>
@@ -4900,7 +4904,7 @@
       </c>
       <c r="C59" s="10"/>
       <c r="D59" s="9">
-        <v>46239.570892222226</v>
+        <v>46255.715298125</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>157</v>
@@ -5055,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="U61" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5067,7 +5071,7 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46239.57100972222</v>
+        <v>46255.71530109954</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>157</v>
@@ -5120,7 +5124,7 @@
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46239.57100552083</v>
+        <v>46255.715298634255</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>157</v>
@@ -5173,7 +5177,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46239.57100167824</v>
+        <v>46255.71529912037</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>157</v>
@@ -5375,7 +5379,7 @@
         <v>0</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5438,7 +5442,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5611,7 +5615,7 @@
         <v>0</v>
       </c>
       <c r="U71" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5886,7 +5890,7 @@
         <v>0</v>
       </c>
       <c r="U76" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6161,7 +6165,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6173,7 +6177,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46239.61779259259</v>
+        <v>46255.71529939814</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>157</v>
@@ -6226,7 +6230,7 @@
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46239.617791365745</v>
+        <v>46255.7152997338</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>157</v>
@@ -6436,7 +6440,7 @@
         <v>0</v>
       </c>
       <c r="U86" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6711,7 +6715,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -6986,7 +6990,7 @@
         <v>0</v>
       </c>
       <c r="U96" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -7261,7 +7265,7 @@
         <v>0</v>
       </c>
       <c r="U101" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
@@ -7583,7 +7587,7 @@
         <v>0</v>
       </c>
       <c r="U107" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
@@ -7858,7 +7862,7 @@
         <v>0</v>
       </c>
       <c r="U112" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
@@ -8131,7 +8135,7 @@
         <v>0</v>
       </c>
       <c r="U117" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
@@ -8406,7 +8410,7 @@
         <v>0</v>
       </c>
       <c r="U122" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
@@ -8728,7 +8732,7 @@
         <v>0</v>
       </c>
       <c r="U128" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
@@ -8791,7 +8795,7 @@
         <v>0</v>
       </c>
       <c r="U129" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>